<commit_message>
new patches regsarding cache
</commit_message>
<xml_diff>
--- a/data/isin_largecap.xlsx
+++ b/data/isin_largecap.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ee1cb525f3e58a26/Desktop/dreamladder/Mutual funds historical analysis/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\utkarsh\OneDrive\Desktop\dreamladder\Mutual funds historical analysis\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{61272646-8C77-4C88-83B9-2F5CC4198625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A57503A-6705-4664-9886-5A2CA3A24392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{02394B5D-3993-4F93-98AB-183138D5C892}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{02394B5D-3993-4F93-98AB-183138D5C892}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="69">
   <si>
     <t xml:space="preserve">Fund name </t>
   </si>
@@ -190,9 +190,6 @@
   </si>
   <si>
     <t>ITI Large Cap Fund (G)</t>
-  </si>
-  <si>
-    <t>JM Large Cap Fund - (G)</t>
   </si>
   <si>
     <t>Kotak Large Cap Fund (G)</t>
@@ -749,7 +746,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>19</v>
@@ -757,7 +754,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>20</v>
@@ -765,7 +762,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>21</v>
@@ -773,7 +770,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>22</v>
@@ -781,7 +778,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>23</v>
@@ -789,7 +786,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>24</v>
@@ -797,7 +794,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>25</v>
@@ -805,7 +802,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>26</v>
@@ -813,7 +810,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>27</v>
@@ -821,7 +818,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>28</v>
@@ -829,7 +826,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>29</v>
@@ -837,7 +834,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>30</v>
@@ -845,7 +842,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>31</v>
@@ -853,7 +850,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>32</v>
@@ -861,7 +858,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>33</v>
@@ -869,7 +866,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>34</v>
@@ -877,7 +874,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>35</v>
@@ -885,7 +882,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>2</v>

</xml_diff>